<commit_message>
Update localization package and UT
</commit_message>
<xml_diff>
--- a/src/main/resources/localization.xlsx
+++ b/src/main/resources/localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hiryu\IdeaProjects\SEP2\javashoppingcartwithlocalizationUIDB\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9E07AE-6743-40D3-8867-9A0EEF4B52A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9108738A-37CE-4E4A-9D8B-3B0C0B23D8CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5A556367-D41A-408F-B5E9-FBDE220F8F23}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="10368" xr2:uid="{5A556367-D41A-408F-B5E9-FBDE220F8F23}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL" sheetId="1" r:id="rId1"/>
@@ -842,7 +842,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1162,7 +1162,7 @@
   <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="23.3984375" customWidth="1"/>
+    <col min="1" max="7" width="19.19921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -1211,7 +1211,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>34</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>55</v>
       </c>

</xml_diff>